<commit_message>
Changed config.py to use a toml
</commit_message>
<xml_diff>
--- a/etc/Archimedes Density TiAg.xlsx
+++ b/etc/Archimedes Density TiAg.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ohp460\Documents\Code\ampm-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ohp460\Documents\Code\ampm-analysis\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8685282E-057F-47B3-BB2D-B8E35237BBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C648635C-B90E-4537-9017-E10ED3D9C175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{29DB1FB1-494D-1A44-8969-5057E69FAAE0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="3" xr2:uid="{29DB1FB1-494D-1A44-8969-5057E69FAAE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Ti-6Ag" sheetId="2" r:id="rId1"/>
     <sheet name="Ti-15Ag" sheetId="3" r:id="rId2"/>
     <sheet name="Ti-25Ag" sheetId="1" r:id="rId3"/>
     <sheet name="Ti-Sterling" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
+    <sheet name="Ti-0.5Cu" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="26">
   <si>
     <t>Energy Density (J/m)</t>
   </si>
@@ -1559,49 +1559,49 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="15"/>
                   <c:pt idx="0">
-                    <c:v>3.410763355418648E-2</c:v>
+                    <c:v>8.2613558209290363E-3</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>1.7337550768971356E-2</c:v>
+                    <c:v>7.5434298123156704E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.1086688715151673E-2</c:v>
+                    <c:v>3.2316146634977193E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>2.773286858584937E-2</c:v>
+                    <c:v>1.6277080000212874E-2</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>2.5207598060902184E-2</c:v>
+                    <c:v>2.8865723618159717E-2</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>2.0128329952250616E-2</c:v>
+                    <c:v>2.7310620644723553E-2</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8271569936363053E-2</c:v>
+                    <c:v>3.1303247967796051E-2</c:v>
                   </c:pt>
                   <c:pt idx="7">
-                    <c:v>3.0706611665893575E-2</c:v>
+                    <c:v>2.5276537210095221E-2</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>1.4827103560709433E-2</c:v>
+                    <c:v>1.8112518691041829E-2</c:v>
                   </c:pt>
                   <c:pt idx="9">
-                    <c:v>2.6363288869182953E-2</c:v>
+                    <c:v>2.0005332622411619E-2</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.2872341375556528E-2</c:v>
+                    <c:v>2.8976542236781724E-2</c:v>
                   </c:pt>
                   <c:pt idx="11">
-                    <c:v>2.2021966306395128E-2</c:v>
+                    <c:v>2.5343243675583403E-2</c:v>
                   </c:pt>
                   <c:pt idx="12">
-                    <c:v>2.0245855542966415E-2</c:v>
+                    <c:v>3.0453297577328651E-2</c:v>
                   </c:pt>
                   <c:pt idx="13">
-                    <c:v>1.5394241347551508E-2</c:v>
+                    <c:v>1.0900611603636284E-2</c:v>
                   </c:pt>
                   <c:pt idx="14">
-                    <c:v>2.6798208895372138E-2</c:v>
+                    <c:v>3.9466568130507806E-2</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1613,49 +1613,49 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="15"/>
                   <c:pt idx="0">
-                    <c:v>3.410763355418648E-2</c:v>
+                    <c:v>8.2613558209290363E-3</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>1.7337550768971356E-2</c:v>
+                    <c:v>7.5434298123156704E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.1086688715151673E-2</c:v>
+                    <c:v>3.2316146634977193E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>2.773286858584937E-2</c:v>
+                    <c:v>1.6277080000212874E-2</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>2.5207598060902184E-2</c:v>
+                    <c:v>2.8865723618159717E-2</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>2.0128329952250616E-2</c:v>
+                    <c:v>2.7310620644723553E-2</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8271569936363053E-2</c:v>
+                    <c:v>3.1303247967796051E-2</c:v>
                   </c:pt>
                   <c:pt idx="7">
-                    <c:v>3.0706611665893575E-2</c:v>
+                    <c:v>2.5276537210095221E-2</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>1.4827103560709433E-2</c:v>
+                    <c:v>1.8112518691041829E-2</c:v>
                   </c:pt>
                   <c:pt idx="9">
-                    <c:v>2.6363288869182953E-2</c:v>
+                    <c:v>2.0005332622411619E-2</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.2872341375556528E-2</c:v>
+                    <c:v>2.8976542236781724E-2</c:v>
                   </c:pt>
                   <c:pt idx="11">
-                    <c:v>2.2021966306395128E-2</c:v>
+                    <c:v>2.5343243675583403E-2</c:v>
                   </c:pt>
                   <c:pt idx="12">
-                    <c:v>2.0245855542966415E-2</c:v>
+                    <c:v>3.0453297577328651E-2</c:v>
                   </c:pt>
                   <c:pt idx="13">
-                    <c:v>1.5394241347551508E-2</c:v>
+                    <c:v>1.0900611603636284E-2</c:v>
                   </c:pt>
                   <c:pt idx="14">
-                    <c:v>2.6798208895372138E-2</c:v>
+                    <c:v>3.9466568130507806E-2</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1755,49 +1755,49 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>4.8771333333333331</c:v>
+                  <c:v>4.9010000000000007</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.8750333333333336</c:v>
+                  <c:v>4.8889333333333331</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8749666666666682</c:v>
+                  <c:v>4.883866666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8570000000000002</c:v>
+                  <c:v>4.8782666666666659</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.8389499999999996</c:v>
+                  <c:v>4.8529000000000009</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.8355166666666669</c:v>
+                  <c:v>4.8388999999999998</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.8305833333333332</c:v>
+                  <c:v>4.847833333333333</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8194999999999988</c:v>
+                  <c:v>4.8431666666666668</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8168499999999996</c:v>
+                  <c:v>4.8104666666666667</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.8000499999999997</c:v>
+                  <c:v>4.8163666666666662</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4.7827999999999999</c:v>
+                  <c:v>4.7923</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.78085</c:v>
+                  <c:v>4.7759</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.7573333333333325</c:v>
+                  <c:v>4.7552666666666665</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.6725333333333339</c:v>
+                  <c:v>4.6808333333333332</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.6513</c:v>
+                  <c:v>4.6478999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2228,49 +2228,49 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="15"/>
                   <c:pt idx="0">
-                    <c:v>3.410763355418648E-2</c:v>
+                    <c:v>8.2613558209290363E-3</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>1.7337550768971356E-2</c:v>
+                    <c:v>7.5434298123156704E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.1086688715151673E-2</c:v>
+                    <c:v>3.2316146634977193E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>2.773286858584937E-2</c:v>
+                    <c:v>1.6277080000212874E-2</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>2.5207598060902184E-2</c:v>
+                    <c:v>2.8865723618159717E-2</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>2.0128329952250616E-2</c:v>
+                    <c:v>2.7310620644723553E-2</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8271569936363053E-2</c:v>
+                    <c:v>3.1303247967796051E-2</c:v>
                   </c:pt>
                   <c:pt idx="7">
-                    <c:v>3.0706611665893575E-2</c:v>
+                    <c:v>2.5276537210095221E-2</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>1.4827103560709433E-2</c:v>
+                    <c:v>1.8112518691041829E-2</c:v>
                   </c:pt>
                   <c:pt idx="9">
-                    <c:v>2.6363288869182953E-2</c:v>
+                    <c:v>2.0005332622411619E-2</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.2872341375556528E-2</c:v>
+                    <c:v>2.8976542236781724E-2</c:v>
                   </c:pt>
                   <c:pt idx="11">
-                    <c:v>2.2021966306395128E-2</c:v>
+                    <c:v>2.5343243675583403E-2</c:v>
                   </c:pt>
                   <c:pt idx="12">
-                    <c:v>2.0245855542966415E-2</c:v>
+                    <c:v>3.0453297577328651E-2</c:v>
                   </c:pt>
                   <c:pt idx="13">
-                    <c:v>1.5394241347551508E-2</c:v>
+                    <c:v>1.0900611603636284E-2</c:v>
                   </c:pt>
                   <c:pt idx="14">
-                    <c:v>2.6798208895372138E-2</c:v>
+                    <c:v>3.9466568130507806E-2</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -2282,49 +2282,49 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="15"/>
                   <c:pt idx="0">
-                    <c:v>3.410763355418648E-2</c:v>
+                    <c:v>8.2613558209290363E-3</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>1.7337550768971356E-2</c:v>
+                    <c:v>7.5434298123156704E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.1086688715151673E-2</c:v>
+                    <c:v>3.2316146634977193E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>2.773286858584937E-2</c:v>
+                    <c:v>1.6277080000212874E-2</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>2.5207598060902184E-2</c:v>
+                    <c:v>2.8865723618159717E-2</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>2.0128329952250616E-2</c:v>
+                    <c:v>2.7310620644723553E-2</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8271569936363053E-2</c:v>
+                    <c:v>3.1303247967796051E-2</c:v>
                   </c:pt>
                   <c:pt idx="7">
-                    <c:v>3.0706611665893575E-2</c:v>
+                    <c:v>2.5276537210095221E-2</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>1.4827103560709433E-2</c:v>
+                    <c:v>1.8112518691041829E-2</c:v>
                   </c:pt>
                   <c:pt idx="9">
-                    <c:v>2.6363288869182953E-2</c:v>
+                    <c:v>2.0005332622411619E-2</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.2872341375556528E-2</c:v>
+                    <c:v>2.8976542236781724E-2</c:v>
                   </c:pt>
                   <c:pt idx="11">
-                    <c:v>2.2021966306395128E-2</c:v>
+                    <c:v>2.5343243675583403E-2</c:v>
                   </c:pt>
                   <c:pt idx="12">
-                    <c:v>2.0245855542966415E-2</c:v>
+                    <c:v>3.0453297577328651E-2</c:v>
                   </c:pt>
                   <c:pt idx="13">
-                    <c:v>1.5394241347551508E-2</c:v>
+                    <c:v>1.0900611603636284E-2</c:v>
                   </c:pt>
                   <c:pt idx="14">
-                    <c:v>2.6798208895372138E-2</c:v>
+                    <c:v>3.9466568130507806E-2</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -2424,49 +2424,49 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>4.8771333333333331</c:v>
+                  <c:v>4.9010000000000007</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.8750333333333336</c:v>
+                  <c:v>4.8889333333333331</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8749666666666682</c:v>
+                  <c:v>4.883866666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8570000000000002</c:v>
+                  <c:v>4.8782666666666659</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.8389499999999996</c:v>
+                  <c:v>4.8529000000000009</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.8355166666666669</c:v>
+                  <c:v>4.8388999999999998</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.8305833333333332</c:v>
+                  <c:v>4.847833333333333</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.8194999999999988</c:v>
+                  <c:v>4.8431666666666668</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8168499999999996</c:v>
+                  <c:v>4.8104666666666667</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.8000499999999997</c:v>
+                  <c:v>4.8163666666666662</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4.7827999999999999</c:v>
+                  <c:v>4.7923</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.78085</c:v>
+                  <c:v>4.7759</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.7573333333333325</c:v>
+                  <c:v>4.7552666666666665</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.6725333333333339</c:v>
+                  <c:v>4.6808333333333332</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.6513</c:v>
+                  <c:v>4.6478999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2895,7 +2895,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AB8CD2F4-8BB3-4469-9EC7-4776F5AD4A29}" type="CELLRANGE">
+                    <a:fld id="{B334CC00-1036-4C95-9C3E-1007016BCC79}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2927,7 +2927,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A9C9690D-D5FB-40B9-9D2C-F6CE17F44446}" type="CELLRANGE">
+                    <a:fld id="{D53C041C-DC98-4838-AB99-3FD1E91284FD}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2960,7 +2960,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AEE56F86-D8E3-4632-8523-526C796683E6}" type="CELLRANGE">
+                    <a:fld id="{52C9BC74-8F11-4F7C-8BDC-11B1AB261B88}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2993,7 +2993,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A8CB8E21-1683-45D0-9337-77EC91C373AC}" type="CELLRANGE">
+                    <a:fld id="{04A33094-0526-4F15-A87C-A250C76FBEA1}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3026,7 +3026,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6EB8186D-5F48-47CA-B665-E037D0ADF8B2}" type="CELLRANGE">
+                    <a:fld id="{00312552-9F01-4F79-9BDC-3B545BC7D539}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3059,7 +3059,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6B7390A4-3EEF-4E2B-830A-2E8678653ECA}" type="CELLRANGE">
+                    <a:fld id="{65B86E88-B456-4969-9905-5E8A5912016A}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3092,7 +3092,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9F4E7711-0A40-491B-87B7-CF4E7C05C945}" type="CELLRANGE">
+                    <a:fld id="{66B2D97E-370C-45A7-ABE0-CA204B6729C1}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3125,7 +3125,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FDE85148-7E18-43FD-9CDB-445A7B2EA3D6}" type="CELLRANGE">
+                    <a:fld id="{7CE0E133-4E30-41C0-91C2-F4CE9C5982C4}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3158,7 +3158,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C137BCE9-4403-4A5C-B60C-2FC5805CB255}" type="CELLRANGE">
+                    <a:fld id="{E3E2187A-125B-434F-83FF-390FCFBDC88F}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3191,7 +3191,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{50B9C386-474D-4207-A892-52CCC2171FDE}" type="CELLRANGE">
+                    <a:fld id="{9946B900-54C0-4CFB-B827-937EDC3CDB5E}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3224,7 +3224,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A136261D-B906-416B-80E0-AD8049B418A7}" type="CELLRANGE">
+                    <a:fld id="{3C45D4B5-9B24-439F-A9F6-0690EC10D480}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3257,7 +3257,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D55ECBCE-419C-4DA6-9572-65807FF1C8A3}" type="CELLRANGE">
+                    <a:fld id="{C8EB616B-081A-40BE-B019-37E3A0B5F8DB}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3290,7 +3290,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2DE4C29A-2BA2-41B3-9CB6-C8B2BDBF9C6F}" type="CELLRANGE">
+                    <a:fld id="{74600BDA-6A65-40E0-A4E8-2383C95261FE}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3323,7 +3323,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DF56B4B4-0243-4CD6-80DD-14CE070CA64A}" type="CELLRANGE">
+                    <a:fld id="{502786ED-65CD-4F42-A252-A58FC6078DEA}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3356,7 +3356,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B8096CC6-CA66-4F4C-9212-5AB50D3A69CF}" type="CELLRANGE">
+                    <a:fld id="{4DED950D-4D24-4E4C-AAC6-555318D81FB0}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3389,7 +3389,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EF6F04C1-C78A-4605-828F-D44BE243CF6A}" type="CELLRANGE">
+                    <a:fld id="{C410097E-E07E-46CF-AF50-75E933C3CF10}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3422,7 +3422,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{89F018E5-C37F-4D45-83C0-3A977921FA51}" type="CELLRANGE">
+                    <a:fld id="{EE419D1E-280A-460E-AD81-23D297309FAB}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3523,7 +3523,7 @@
                     <c:v>4.8751068364363817E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.0214368964029757E-2</c:v>
+                    <c:v>4.0414518843273749E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
                     <c:v>4.0414518843273749E-3</c:v>
@@ -3589,7 +3589,7 @@
                     <c:v>4.8751068364363817E-3</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>1.0214368964029757E-2</c:v>
+                    <c:v>4.0414518843273749E-3</c:v>
                   </c:pt>
                   <c:pt idx="3">
                     <c:v>4.0414518843273749E-3</c:v>
@@ -3729,7 +3729,7 @@
                   <c:v>4.8031666666666668</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8406666666666665</c:v>
+                  <c:v>4.8486666666666665</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>4.839666666666667</c:v>
@@ -27635,12 +27635,12 @@
         <v>116.66666666666667</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E16" si="1">AVERAGE(G2:L2)</f>
-        <v>4.8771333333333331</v>
+        <f t="shared" ref="E2:E16" si="1">AVERAGE(J2:L2)</f>
+        <v>4.9010000000000007</v>
       </c>
       <c r="F2">
-        <f t="shared" ref="F2:F16" si="2">STDEV(G2:L2)</f>
-        <v>3.410763355418648E-2</v>
+        <f t="shared" ref="F2:F16" si="2">STDEV(J2:L2)</f>
+        <v>8.2613558209290363E-3</v>
       </c>
       <c r="G2" s="1">
         <v>4.8174000000000001</v>
@@ -27680,11 +27680,11 @@
       </c>
       <c r="E3" s="1">
         <f t="shared" si="1"/>
-        <v>4.8750333333333336</v>
+        <v>4.8889333333333331</v>
       </c>
       <c r="F3">
         <f t="shared" si="2"/>
-        <v>1.7337550768971356E-2</v>
+        <v>7.5434298123156704E-3</v>
       </c>
       <c r="G3" s="1">
         <v>4.8701999999999996</v>
@@ -27724,11 +27724,11 @@
       </c>
       <c r="E4" s="1">
         <f t="shared" si="1"/>
-        <v>4.8749666666666682</v>
+        <v>4.883866666666667</v>
       </c>
       <c r="F4">
         <f t="shared" si="2"/>
-        <v>1.1086688715151673E-2</v>
+        <v>3.2316146634977193E-3</v>
       </c>
       <c r="G4" s="1">
         <v>4.8571999999999997</v>
@@ -27768,11 +27768,11 @@
       </c>
       <c r="E5" s="1">
         <f t="shared" si="1"/>
-        <v>4.8570000000000002</v>
+        <v>4.8782666666666659</v>
       </c>
       <c r="F5">
         <f t="shared" si="2"/>
-        <v>2.773286858584937E-2</v>
+        <v>1.6277080000212874E-2</v>
       </c>
       <c r="G5" s="1">
         <v>4.8219000000000003</v>
@@ -27812,11 +27812,11 @@
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
-        <v>4.8389499999999996</v>
+        <v>4.8529000000000009</v>
       </c>
       <c r="F6">
         <f t="shared" si="2"/>
-        <v>2.5207598060902184E-2</v>
+        <v>2.8865723618159717E-2</v>
       </c>
       <c r="G6" s="1">
         <v>4.8217999999999996</v>
@@ -27854,11 +27854,11 @@
       </c>
       <c r="E7" s="1">
         <f t="shared" si="1"/>
-        <v>4.8355166666666669</v>
+        <v>4.8388999999999998</v>
       </c>
       <c r="F7">
         <f t="shared" si="2"/>
-        <v>2.0128329952250616E-2</v>
+        <v>2.7310620644723553E-2</v>
       </c>
       <c r="G7" s="1">
         <v>4.8148999999999997</v>
@@ -27898,11 +27898,11 @@
       </c>
       <c r="E8" s="1">
         <f t="shared" si="1"/>
-        <v>4.8305833333333332</v>
+        <v>4.847833333333333</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>2.8271569936363053E-2</v>
+        <v>3.1303247967796051E-2</v>
       </c>
       <c r="G8" s="1">
         <v>4.8232999999999997</v>
@@ -27940,11 +27940,11 @@
       </c>
       <c r="E9" s="1">
         <f t="shared" si="1"/>
-        <v>4.8194999999999988</v>
+        <v>4.8431666666666668</v>
       </c>
       <c r="F9">
         <f t="shared" si="2"/>
-        <v>3.0706611665893575E-2</v>
+        <v>2.5276537210095221E-2</v>
       </c>
       <c r="G9" s="1">
         <v>4.7972000000000001</v>
@@ -27982,11 +27982,11 @@
       </c>
       <c r="E10" s="1">
         <f t="shared" si="1"/>
-        <v>4.8168499999999996</v>
+        <v>4.8104666666666667</v>
       </c>
       <c r="F10">
         <f t="shared" si="2"/>
-        <v>1.4827103560709433E-2</v>
+        <v>1.8112518691041829E-2</v>
       </c>
       <c r="G10" s="1">
         <v>4.8190999999999997</v>
@@ -28024,11 +28024,11 @@
       </c>
       <c r="E11" s="1">
         <f t="shared" si="1"/>
-        <v>4.8000499999999997</v>
+        <v>4.8163666666666662</v>
       </c>
       <c r="F11">
         <f t="shared" si="2"/>
-        <v>2.6363288869182953E-2</v>
+        <v>2.0005332622411619E-2</v>
       </c>
       <c r="G11" s="1">
         <v>4.7830000000000004</v>
@@ -28068,11 +28068,11 @@
       </c>
       <c r="E12" s="1">
         <f t="shared" si="1"/>
-        <v>4.7827999999999999</v>
+        <v>4.7923</v>
       </c>
       <c r="F12">
         <f t="shared" si="2"/>
-        <v>2.2872341375556528E-2</v>
+        <v>2.8976542236781724E-2</v>
       </c>
       <c r="G12" s="1">
         <v>4.7805999999999997</v>
@@ -28110,11 +28110,11 @@
       </c>
       <c r="E13" s="1">
         <f t="shared" si="1"/>
-        <v>4.78085</v>
+        <v>4.7759</v>
       </c>
       <c r="F13">
         <f t="shared" si="2"/>
-        <v>2.2021966306395128E-2</v>
+        <v>2.5343243675583403E-2</v>
       </c>
       <c r="G13" s="1">
         <v>4.7797000000000001</v>
@@ -28152,11 +28152,11 @@
       </c>
       <c r="E14" s="1">
         <f t="shared" si="1"/>
-        <v>4.7573333333333325</v>
+        <v>4.7552666666666665</v>
       </c>
       <c r="F14">
         <f t="shared" si="2"/>
-        <v>2.0245855542966415E-2</v>
+        <v>3.0453297577328651E-2</v>
       </c>
       <c r="G14" s="1">
         <v>4.7535999999999996</v>
@@ -28194,11 +28194,11 @@
       </c>
       <c r="E15" s="1">
         <f t="shared" si="1"/>
-        <v>4.6725333333333339</v>
+        <v>4.6808333333333332</v>
       </c>
       <c r="F15">
         <f t="shared" si="2"/>
-        <v>1.5394241347551508E-2</v>
+        <v>1.0900611603636284E-2</v>
       </c>
       <c r="G15" s="1">
         <v>4.6470000000000002</v>
@@ -28236,11 +28236,11 @@
       </c>
       <c r="E16" s="1">
         <f t="shared" si="1"/>
-        <v>4.6513</v>
+        <v>4.6478999999999999</v>
       </c>
       <c r="F16">
         <f t="shared" si="2"/>
-        <v>2.6798208895372138E-2</v>
+        <v>3.9466568130507806E-2</v>
       </c>
       <c r="G16" s="1">
         <v>4.6405000000000003</v>
@@ -28523,20 +28523,20 @@
       </c>
       <c r="E4" s="1">
         <f t="shared" si="1"/>
-        <v>4.8406666666666665</v>
+        <v>4.8486666666666665</v>
       </c>
       <c r="F4" s="9">
         <f t="shared" ref="F4:F16" si="2">STDEV(G4:I4)</f>
-        <v>1.0214368964029757E-2</v>
+        <v>4.0414518843273749E-3</v>
       </c>
       <c r="G4" s="7">
-        <v>4.8289999999999997</v>
+        <v>4.8479999999999999</v>
       </c>
       <c r="H4" s="8">
         <v>4.8449999999999998</v>
       </c>
       <c r="I4" s="8">
-        <v>4.8479999999999999</v>
+        <v>4.8529999999999998</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
@@ -29147,6 +29147,9 @@
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
       <c r="B1" t="s">
         <v>13</v>
       </c>
@@ -29162,7 +29165,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4.5990000000000002</v>
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="C2">
+        <v>4.5220000000000002</v>
+      </c>
+      <c r="D2">
+        <v>4.5179999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
@@ -29170,7 +29179,13 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4.6079999999999997</v>
+        <v>4.5220000000000002</v>
+      </c>
+      <c r="C3">
+        <v>4.5229999999999997</v>
+      </c>
+      <c r="D3">
+        <v>4.5199999999999996</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
@@ -29178,7 +29193,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>4.6050000000000004</v>
+        <v>4.524</v>
+      </c>
+      <c r="C4">
+        <v>4.5229999999999997</v>
+      </c>
+      <c r="D4">
+        <v>4.5209999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
@@ -29186,7 +29207,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>4.6050000000000004</v>
+        <v>4.5209999999999999</v>
+      </c>
+      <c r="C5">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="D5">
+        <v>4.5209999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
@@ -29194,7 +29221,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>4.601</v>
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="C6">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="D6">
+        <v>4.5190000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -29202,7 +29235,13 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>4.6029999999999998</v>
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="C7">
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="D7">
+        <v>4.5209999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -29210,7 +29249,13 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>4.5999999999999996</v>
+        <v>4.5179999999999998</v>
+      </c>
+      <c r="C8">
+        <v>4.5209999999999999</v>
+      </c>
+      <c r="D8">
+        <v>4.5209999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
@@ -29218,7 +29263,13 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>4.5990000000000002</v>
+        <v>4.5179999999999998</v>
+      </c>
+      <c r="C9">
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="D9">
+        <v>4.5190000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
@@ -29226,7 +29277,13 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>4.5990000000000002</v>
+        <v>4.5190000000000001</v>
+      </c>
+      <c r="C10">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="D10">
+        <v>4.5209999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
@@ -29234,7 +29291,13 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>4.5990000000000002</v>
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="C11">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="D11">
+        <v>4.5179999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>